<commit_message>
Testes com utentes dia 1
</commit_message>
<xml_diff>
--- a/tabelas_utentes/back_scratch_utentes.xlsx
+++ b/tabelas_utentes/back_scratch_utentes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1693,15 +1693,11 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>77</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1.50</t>
-        </is>
+      <c r="A49" t="n">
+        <v>77</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1.5</v>
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
@@ -1712,17 +1708,645 @@
       <c r="E49" t="n">
         <v>-18</v>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>-18.37</t>
-        </is>
+      <c r="F49" t="n">
+        <v>-18.37</v>
       </c>
       <c r="G49" t="n">
         <v>0.370000000000001</v>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>56</t>
+      <c r="H49" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>72</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H50" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>72</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>-3.09</v>
+      </c>
+      <c r="G51" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H51" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>72</v>
+      </c>
+      <c r="B52" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>-15</v>
+      </c>
+      <c r="F52" t="n">
+        <v>-16</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>72</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>-15</v>
+      </c>
+      <c r="F53" t="n">
+        <v>-16.26</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1.260000000000002</v>
+      </c>
+      <c r="H53" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>72</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>-8.26</v>
+      </c>
+      <c r="G54" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="H54" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>72</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-7.46</v>
+      </c>
+      <c r="G55" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="H55" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>72</v>
+      </c>
+      <c r="B56" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>-5</v>
+      </c>
+      <c r="F56" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="G56" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H56" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>72</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F57" t="n">
+        <v>-1.91</v>
+      </c>
+      <c r="G57" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="H57" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>71</v>
+      </c>
+      <c r="B58" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>-15</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-14.06</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.9399999999999995</v>
+      </c>
+      <c r="H58" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>71</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>-23</v>
+      </c>
+      <c r="F59" t="n">
+        <v>-21</v>
+      </c>
+      <c r="G59" t="n">
+        <v>2</v>
+      </c>
+      <c r="H59" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>71</v>
+      </c>
+      <c r="B60" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>-21</v>
+      </c>
+      <c r="F60" t="n">
+        <v>-10</v>
+      </c>
+      <c r="G60" t="n">
+        <v>11</v>
+      </c>
+      <c r="H60" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>71</v>
+      </c>
+      <c r="B61" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>-22.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>-23.86</v>
+      </c>
+      <c r="G61" t="n">
+        <v>1.359999999999999</v>
+      </c>
+      <c r="H61" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>71</v>
+      </c>
+      <c r="B62" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>-16.7</v>
+      </c>
+      <c r="F62" t="n">
+        <v>-16.12</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.5799999999999983</v>
+      </c>
+      <c r="H62" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>71</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>-16</v>
+      </c>
+      <c r="F63" t="n">
+        <v>-14.59</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H63" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>71</v>
+      </c>
+      <c r="B64" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>-22</v>
+      </c>
+      <c r="F64" t="n">
+        <v>-21.85</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.1499999999999986</v>
+      </c>
+      <c r="H64" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>71</v>
+      </c>
+      <c r="B65" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>-20</v>
+      </c>
+      <c r="F65" t="n">
+        <v>-18.5</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H65" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>66</v>
+      </c>
+      <c r="B66" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>-0.74</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="H66" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="G67" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="H67" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H68" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>66</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="H69" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>-3.13</v>
+      </c>
+      <c r="G70" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="H70" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>66</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0</v>
+      </c>
+      <c r="F71" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H71" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>66</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" t="n">
+        <v>-3.09</v>
+      </c>
+      <c r="G72" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H72" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>-0.34</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Testes com utentes dia 2
</commit_message>
<xml_diff>
--- a/tabelas_utentes/back_scratch_utentes.xlsx
+++ b/tabelas_utentes/back_scratch_utentes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2317,15 +2317,11 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
+      <c r="A73" t="n">
+        <v>66</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1.54</v>
       </c>
       <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
@@ -2336,17 +2332,229 @@
       <c r="E73" t="n">
         <v>0</v>
       </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>-0.34</t>
-        </is>
+      <c r="F73" t="n">
+        <v>-0.34</v>
       </c>
       <c r="G73" t="n">
         <v>0.34</v>
       </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>50</t>
+      <c r="H73" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>71</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>-11</v>
+      </c>
+      <c r="F74" t="n">
+        <v>-9.98</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="H74" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>-13</v>
+      </c>
+      <c r="F75" t="n">
+        <v>-10.65</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="H75" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>71</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>-21</v>
+      </c>
+      <c r="F76" t="n">
+        <v>-22.59</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="H76" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>71</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>-14</v>
+      </c>
+      <c r="F77" t="n">
+        <v>-12.59</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="H77" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>71</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>-13</v>
+      </c>
+      <c r="F78" t="n">
+        <v>-13.71</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0.7100000000000009</v>
+      </c>
+      <c r="H78" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>71</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>-14</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-12.37</v>
+      </c>
+      <c r="G79" t="n">
+        <v>1.630000000000001</v>
+      </c>
+      <c r="H79" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>71</v>
+      </c>
+      <c r="B80" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>-16</v>
+      </c>
+      <c r="F80" t="n">
+        <v>-13.91</v>
+      </c>
+      <c r="G80" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="H80" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>-18</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>-15.60</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>75</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Testes com utentens dia 3
</commit_message>
<xml_diff>
--- a/tabelas_utentes/back_scratch_utentes.xlsx
+++ b/tabelas_utentes/back_scratch_utentes.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="10">
   <si>
     <t>Age</t>
   </si>
@@ -457,7 +457,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -3353,10 +3353,10 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
-      <c r="A121" s="7">
+      <c r="A121" s="4">
         <v>73</v>
       </c>
-      <c r="B121" s="8">
+      <c r="B121" s="5">
         <v>1.66</v>
       </c>
       <c r="C121" s="6"/>
@@ -3366,14 +3366,206 @@
       <c r="E121" s="4">
         <v>-17</v>
       </c>
-      <c r="F121" s="8">
+      <c r="F121" s="5">
         <v>-18.43</v>
       </c>
       <c r="G121" s="5">
         <v>1.43</v>
       </c>
-      <c r="H121" s="7">
+      <c r="H121" s="4">
         <v>68</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+      <c r="A122" s="4">
+        <v>82</v>
+      </c>
+      <c r="B122" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C122" s="6"/>
+      <c r="D122" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E122" s="4">
+        <v>-31</v>
+      </c>
+      <c r="F122" s="5">
+        <v>-32.91</v>
+      </c>
+      <c r="G122" s="5">
+        <v>1.91</v>
+      </c>
+      <c r="H122" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+      <c r="A123" s="4">
+        <v>82</v>
+      </c>
+      <c r="B123" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C123" s="6"/>
+      <c r="D123" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E123" s="4">
+        <v>-27</v>
+      </c>
+      <c r="F123" s="5">
+        <v>-30.86</v>
+      </c>
+      <c r="G123" s="5">
+        <v>3.86</v>
+      </c>
+      <c r="H123" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+      <c r="A124" s="4">
+        <v>82</v>
+      </c>
+      <c r="B124" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C124" s="6"/>
+      <c r="D124" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E124" s="4">
+        <v>-32</v>
+      </c>
+      <c r="F124" s="5">
+        <v>-30.29</v>
+      </c>
+      <c r="G124" s="5">
+        <v>1.71</v>
+      </c>
+      <c r="H124" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+      <c r="A125" s="4">
+        <v>82</v>
+      </c>
+      <c r="B125" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C125" s="6"/>
+      <c r="D125" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E125" s="4">
+        <v>-40</v>
+      </c>
+      <c r="F125" s="5">
+        <v>-38.72</v>
+      </c>
+      <c r="G125" s="5">
+        <v>1.28</v>
+      </c>
+      <c r="H125" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+      <c r="A126" s="4">
+        <v>82</v>
+      </c>
+      <c r="B126" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C126" s="6"/>
+      <c r="D126" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E126" s="4">
+        <v>-30</v>
+      </c>
+      <c r="F126" s="5">
+        <v>-34.83</v>
+      </c>
+      <c r="G126" s="5">
+        <v>4.83</v>
+      </c>
+      <c r="H126" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+      <c r="A127" s="4">
+        <v>82</v>
+      </c>
+      <c r="B127" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C127" s="6"/>
+      <c r="D127" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E127" s="4">
+        <v>-30</v>
+      </c>
+      <c r="F127" s="5">
+        <v>-27.62</v>
+      </c>
+      <c r="G127" s="5">
+        <v>2.38</v>
+      </c>
+      <c r="H127" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+      <c r="A128" s="4">
+        <v>82</v>
+      </c>
+      <c r="B128" s="5">
+        <v>1.69</v>
+      </c>
+      <c r="C128" s="6"/>
+      <c r="D128" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E128" s="4">
+        <v>-31</v>
+      </c>
+      <c r="F128" s="5">
+        <v>-28.73</v>
+      </c>
+      <c r="G128" s="5">
+        <v>2.27</v>
+      </c>
+      <c r="H128" s="4">
+        <v>81</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+      <c r="A129" s="7">
+        <v>82</v>
+      </c>
+      <c r="B129" s="8">
+        <v>1.69</v>
+      </c>
+      <c r="C129" s="6"/>
+      <c r="D129" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E129" s="4">
+        <v>-42</v>
+      </c>
+      <c r="F129" s="8">
+        <v>-48.52</v>
+      </c>
+      <c r="G129" s="5">
+        <v>6.52</v>
+      </c>
+      <c r="H129" s="7">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>